<commit_message>
Add simple General and SAP validation setup with 200 columns
</commit_message>
<xml_diff>
--- a/validation-setup-template.xlsx
+++ b/validation-setup-template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="Rb8e2f09524c94eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rf5a078aa222344f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R14762db9296d4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="Rbb0b616fb89c44cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R170424af1b9d44f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R274e691ab99f4d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="R3ddaad93b1734feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Ra6a13ac2b33741a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R9d5d93231b164856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rdf0e0141df024f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R8efab30ae9544022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R3f97f1e005b14e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R5876b80466544567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R3f86236627b54cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rd8053f9e33204341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R677617d23d3241ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,6 +308,7 @@
     <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="75" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -320,6 +321,9 @@
       <x:c r="C1" s="6" t="str">
         <x:v>Format version</x:v>
       </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Template type</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -330,6 +334,9 @@
       </x:c>
       <x:c r="C2" s="7" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>General</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -356,6 +363,10 @@
     <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="19" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="45" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="14" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -404,6 +415,18 @@
       <x:c r="O1" s="6" t="str">
         <x:v>Description</x:v>
       </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>SAP type</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>SAP length</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>SAP decimals</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>SAP reference field</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -435,6 +458,10 @@
       <x:c r="O2" s="7" t="str">
         <x:v>Keep identifiers as text to preserve leading zeros.</x:v>
       </x:c>
+      <x:c r="P2" s="7" t="str"/>
+      <x:c r="Q2" s="7" t="str"/>
+      <x:c r="R2" s="7" t="str"/>
+      <x:c r="S2" s="7" t="str"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
@@ -462,6 +489,10 @@
       <x:c r="M3" s="7" t="str"/>
       <x:c r="N3" s="7" t="str"/>
       <x:c r="O3" s="7" t="str"/>
+      <x:c r="P3" s="7" t="str"/>
+      <x:c r="Q3" s="7" t="str"/>
+      <x:c r="R3" s="7" t="str"/>
+      <x:c r="S3" s="7" t="str"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -487,6 +518,10 @@
       <x:c r="M4" s="7" t="str"/>
       <x:c r="N4" s="7" t="str"/>
       <x:c r="O4" s="7" t="str"/>
+      <x:c r="P4" s="7" t="str"/>
+      <x:c r="Q4" s="7" t="str"/>
+      <x:c r="R4" s="7" t="str"/>
+      <x:c r="S4" s="7" t="str"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="7" t="str">
@@ -514,6 +549,10 @@
       <x:c r="M5" s="7" t="str"/>
       <x:c r="N5" s="7" t="str"/>
       <x:c r="O5" s="7" t="str"/>
+      <x:c r="P5" s="7" t="str"/>
+      <x:c r="Q5" s="7" t="str"/>
+      <x:c r="R5" s="7" t="str"/>
+      <x:c r="S5" s="7" t="str"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="7" t="str">
@@ -543,6 +582,10 @@
       <x:c r="M6" s="7" t="str"/>
       <x:c r="N6" s="7" t="str"/>
       <x:c r="O6" s="7" t="str"/>
+      <x:c r="P6" s="7" t="str"/>
+      <x:c r="Q6" s="7" t="str"/>
+      <x:c r="R6" s="7" t="str"/>
+      <x:c r="S6" s="7" t="str"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="7" t="str">
@@ -568,25 +611,29 @@
       <x:c r="M7" s="7" t="str"/>
       <x:c r="N7" s="7" t="str"/>
       <x:c r="O7" s="7" t="str"/>
+      <x:c r="P7" s="7" t="str"/>
+      <x:c r="Q7" s="7" t="str"/>
+      <x:c r="R7" s="7" t="str"/>
+      <x:c r="S7" s="7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="6">
-    <x:dataValidation type="list" sqref="C2:C100">
+    <x:dataValidation type="list" sqref="C2:C201">
       <x:formula1>"text,integer,decimal,date,boolean"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D2:D100">
+    <x:dataValidation type="list" sqref="D2:D201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E2:E100">
+    <x:dataValidation type="list" sqref="E2:E201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="L2:L100">
+    <x:dataValidation type="list" sqref="L2:L201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M2:M100">
+    <x:dataValidation type="list" sqref="M2:M201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="N2:N100">
+    <x:dataValidation type="list" sqref="N2:N201">
       <x:formula1>"digits,alphanumeric,email,url,identifier"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -815,7 +862,7 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="C2:C100">
+    <x:dataValidation type="list" sqref="C2:C201">
       <x:formula1>"error,warning"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D100">
@@ -1051,8 +1098,9 @@
         <x:v>Edit Template, then Columns. Each field uses one row. Header rows must stay in row 1. Delete example rows you do not need.</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Template: one name row. Columns: 1–80 fields.</x:v>
-      </x:c>
+        <x:v>Template: one name row. Columns: 1–200 fields.</x:v>
+      </x:c>
+      <x:c r="D2" s="10"/>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -1064,6 +1112,7 @@
       <x:c r="C3" s="9" t="str">
         <x:v>Your saved templates and published versions are preserved.</x:v>
       </x:c>
+      <x:c r="D3" s="10"/>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -1075,6 +1124,7 @@
       <x:c r="C4" s="9" t="str">
         <x:v>MATERIAL / Material / text</x:v>
       </x:c>
+      <x:c r="D4" s="10"/>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -1086,6 +1136,7 @@
       <x:c r="C5" s="9" t="str">
         <x:v>A blank Min or Max means no limit. Zero is a valid limit.</x:v>
       </x:c>
+      <x:c r="D5" s="10"/>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -1097,6 +1148,7 @@
       <x:c r="C6" s="9" t="str">
         <x:v>Allowed values: 101,201</x:v>
       </x:c>
+      <x:c r="D6" s="10"/>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -1108,6 +1160,7 @@
       <x:c r="C7" s="9" t="str">
         <x:v>identifier allows letters, numbers, underscores and hyphens.</x:v>
       </x:c>
+      <x:c r="D7" s="10"/>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="9" t="str">
@@ -1119,6 +1172,7 @@
       <x:c r="C8" s="9" t="str">
         <x:v>Name, Severity, Enabled and Message can be set on the first row.</x:v>
       </x:c>
+      <x:c r="D8" s="10"/>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="9" t="str">
@@ -1130,6 +1184,7 @@
       <x:c r="C9" s="9" t="str">
         <x:v>Field values must match the exact technical keys from Columns.</x:v>
       </x:c>
+      <x:c r="D9" s="10"/>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="9" t="str">
@@ -1141,6 +1196,7 @@
       <x:c r="C10" s="9" t="str">
         <x:v>Group root / Join all; Group 1 / Join any</x:v>
       </x:c>
+      <x:c r="D10" s="10"/>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="9" t="str">
@@ -1152,6 +1208,7 @@
       <x:c r="C11" s="9" t="str">
         <x:v>MOVEMENT_TYPE / eq / 201</x:v>
       </x:c>
+      <x:c r="D11" s="10"/>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -1163,6 +1220,7 @@
       <x:c r="C12" s="9" t="str">
         <x:v>END_DATE / fieldGte / Other field START_DATE</x:v>
       </x:c>
+      <x:c r="D12" s="10"/>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="9" t="str">
@@ -1174,6 +1232,7 @@
       <x:c r="C13" s="9" t="str">
         <x:v>CONTACT / pattern / email</x:v>
       </x:c>
+      <x:c r="D13" s="10"/>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="9" t="str">
@@ -1185,6 +1244,7 @@
       <x:c r="C14" s="9" t="str">
         <x:v>Separate Description columns with semicolons or newlines.</x:v>
       </x:c>
+      <x:c r="D14" s="10"/>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="9" t="str">
@@ -1196,6 +1256,7 @@
       <x:c r="C15" s="9" t="str">
         <x:v>PLANT / lookup / plants / Plant</x:v>
       </x:c>
+      <x:c r="D15" s="10"/>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="9" t="str">
@@ -1207,6 +1268,7 @@
       <x:c r="C16" s="9" t="str">
         <x:v>PLANT=Plant;STORAGE_LOCATION=Storage location</x:v>
       </x:c>
+      <x:c r="D16" s="10"/>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="9" t="str">
@@ -1218,17 +1280,19 @@
       <x:c r="C17" s="9" t="str">
         <x:v>MATERIAL,PLANT,STORAGE_LOCATION</x:v>
       </x:c>
+      <x:c r="D17" s="10"/>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>Limits</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>Up to 80 columns, 100 rules, 400 when clauses, 20 reference lists and 20 unique combinations. Keep the workbook below 10 MB.</x:v>
+        <x:v>Up to 200 columns, 100 rules, 400 when clauses, 20 reference lists and 20 unique combinations. Keep the workbook below 10 MB.</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
         <x:v>Remove a sheet only when you do not use that section. Template and Columns are required.</x:v>
       </x:c>
+      <x:c r="D18" s="10"/>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="9" t="str">
@@ -1240,11 +1304,63 @@
       <x:c r="C19" s="9" t="str">
         <x:v>This file configures validation rules. Use the Validate tab for data files to check.</x:v>
       </x:c>
+      <x:c r="D19" s="10"/>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
-      <x:c r="A20" s="10"/>
-      <x:c r="B20" s="10"/>
-      <x:c r="C20" s="10"/>
+      <x:c r="A20" s="9" t="str">
+        <x:v>Template type</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>General preserves the existing checks. For SAP choose SAP in Template, and fill SAP type, SAP length, SAP decimals and optional SAP reference field on Columns. General Type stays text if unused.</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="str">
+        <x:v>SAP date DATS / 8; currency CURR / 15 / 2 → CUKY field.</x:v>
+      </x:c>
+      <x:c r="D20" s="10"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="7" t="str">
+        <x:v>SAP formats</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="str">
+        <x:v>Use internal formats: DATS YYYYMMDD (initial 00000000), TIMS HHMMSS, NUMC fixed digits, signed plain decimals with a dot. No zero padding, rounding or conversion exits are applied.</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="str">
+        <x:v>Keep technical codes and long numbers as Text in Excel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="7" t="str">
+        <x:v>SAP scope</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>18 supported DDIC formats. Use actual SE11 definitions. Domain values, conversion exits and currency display scaling need your system-specific Conditions/References.</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Source: https://help.sap.com/doc/abapdocu_754_index_htm/7.54/en-US/abenddic_builtin_types.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="7" t="str">
+        <x:v>Simpler option</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>For column setup without Excel conditions/references, use the one-sheet simple General or SAP setup download instead. You can maintain Conditions and References later inside Studio.</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>A single Setup sheet: name in B2, type in B3, fields from row 9.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="7" t="str">
+        <x:v>Upload size</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="str">
+        <x:v>Data validation stays within 5,000 rows and 200,000 cells. At 200 columns, upload up to 1,000 data rows per file.</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="str">
+        <x:v>Setup rows define fields; data rows are uploaded separately on Validate.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Simplify validation setup and add SAP formats with 200 columns (#101)
* Add simple General and SAP validation setup with 200 columns

* Keep 200-column editor field lists scrollable

* Reject unsupported SAP type names in imported definitions
</commit_message>
<xml_diff>
--- a/validation-setup-template.xlsx
+++ b/validation-setup-template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="Rb8e2f09524c94eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rf5a078aa222344f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R14762db9296d4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="Rbb0b616fb89c44cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R170424af1b9d44f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R274e691ab99f4d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="R3ddaad93b1734feb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="Ra6a13ac2b33741a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R9d5d93231b164856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rdf0e0141df024f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R8efab30ae9544022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R3f97f1e005b14e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R5876b80466544567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R3f86236627b54cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rd8053f9e33204341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R677617d23d3241ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -308,6 +308,7 @@
     <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="75" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -320,6 +321,9 @@
       <x:c r="C1" s="6" t="str">
         <x:v>Format version</x:v>
       </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>Template type</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -330,6 +334,9 @@
       </x:c>
       <x:c r="C2" s="7" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="str">
+        <x:v>General</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -356,6 +363,10 @@
     <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="19" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="45" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="14" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
@@ -404,6 +415,18 @@
       <x:c r="O1" s="6" t="str">
         <x:v>Description</x:v>
       </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>SAP type</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>SAP length</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>SAP decimals</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>SAP reference field</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -435,6 +458,10 @@
       <x:c r="O2" s="7" t="str">
         <x:v>Keep identifiers as text to preserve leading zeros.</x:v>
       </x:c>
+      <x:c r="P2" s="7" t="str"/>
+      <x:c r="Q2" s="7" t="str"/>
+      <x:c r="R2" s="7" t="str"/>
+      <x:c r="S2" s="7" t="str"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="7" t="str">
@@ -462,6 +489,10 @@
       <x:c r="M3" s="7" t="str"/>
       <x:c r="N3" s="7" t="str"/>
       <x:c r="O3" s="7" t="str"/>
+      <x:c r="P3" s="7" t="str"/>
+      <x:c r="Q3" s="7" t="str"/>
+      <x:c r="R3" s="7" t="str"/>
+      <x:c r="S3" s="7" t="str"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="7" t="str">
@@ -487,6 +518,10 @@
       <x:c r="M4" s="7" t="str"/>
       <x:c r="N4" s="7" t="str"/>
       <x:c r="O4" s="7" t="str"/>
+      <x:c r="P4" s="7" t="str"/>
+      <x:c r="Q4" s="7" t="str"/>
+      <x:c r="R4" s="7" t="str"/>
+      <x:c r="S4" s="7" t="str"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="7" t="str">
@@ -514,6 +549,10 @@
       <x:c r="M5" s="7" t="str"/>
       <x:c r="N5" s="7" t="str"/>
       <x:c r="O5" s="7" t="str"/>
+      <x:c r="P5" s="7" t="str"/>
+      <x:c r="Q5" s="7" t="str"/>
+      <x:c r="R5" s="7" t="str"/>
+      <x:c r="S5" s="7" t="str"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="7" t="str">
@@ -543,6 +582,10 @@
       <x:c r="M6" s="7" t="str"/>
       <x:c r="N6" s="7" t="str"/>
       <x:c r="O6" s="7" t="str"/>
+      <x:c r="P6" s="7" t="str"/>
+      <x:c r="Q6" s="7" t="str"/>
+      <x:c r="R6" s="7" t="str"/>
+      <x:c r="S6" s="7" t="str"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="7" t="str">
@@ -568,25 +611,29 @@
       <x:c r="M7" s="7" t="str"/>
       <x:c r="N7" s="7" t="str"/>
       <x:c r="O7" s="7" t="str"/>
+      <x:c r="P7" s="7" t="str"/>
+      <x:c r="Q7" s="7" t="str"/>
+      <x:c r="R7" s="7" t="str"/>
+      <x:c r="S7" s="7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="6">
-    <x:dataValidation type="list" sqref="C2:C100">
+    <x:dataValidation type="list" sqref="C2:C201">
       <x:formula1>"text,integer,decimal,date,boolean"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D2:D100">
+    <x:dataValidation type="list" sqref="D2:D201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E2:E100">
+    <x:dataValidation type="list" sqref="E2:E201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="L2:L100">
+    <x:dataValidation type="list" sqref="L2:L201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M2:M100">
+    <x:dataValidation type="list" sqref="M2:M201">
       <x:formula1>"Yes,No"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="N2:N100">
+    <x:dataValidation type="list" sqref="N2:N201">
       <x:formula1>"digits,alphanumeric,email,url,identifier"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -815,7 +862,7 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="C2:C100">
+    <x:dataValidation type="list" sqref="C2:C201">
       <x:formula1>"error,warning"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D100">
@@ -1051,8 +1098,9 @@
         <x:v>Edit Template, then Columns. Each field uses one row. Header rows must stay in row 1. Delete example rows you do not need.</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Template: one name row. Columns: 1–80 fields.</x:v>
-      </x:c>
+        <x:v>Template: one name row. Columns: 1–200 fields.</x:v>
+      </x:c>
+      <x:c r="D2" s="10"/>
     </x:row>
     <x:row r="3" ht="64" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -1064,6 +1112,7 @@
       <x:c r="C3" s="9" t="str">
         <x:v>Your saved templates and published versions are preserved.</x:v>
       </x:c>
+      <x:c r="D3" s="10"/>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -1075,6 +1124,7 @@
       <x:c r="C4" s="9" t="str">
         <x:v>MATERIAL / Material / text</x:v>
       </x:c>
+      <x:c r="D4" s="10"/>
     </x:row>
     <x:row r="5" ht="64" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -1086,6 +1136,7 @@
       <x:c r="C5" s="9" t="str">
         <x:v>A blank Min or Max means no limit. Zero is a valid limit.</x:v>
       </x:c>
+      <x:c r="D5" s="10"/>
     </x:row>
     <x:row r="6" ht="64" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -1097,6 +1148,7 @@
       <x:c r="C6" s="9" t="str">
         <x:v>Allowed values: 101,201</x:v>
       </x:c>
+      <x:c r="D6" s="10"/>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -1108,6 +1160,7 @@
       <x:c r="C7" s="9" t="str">
         <x:v>identifier allows letters, numbers, underscores and hyphens.</x:v>
       </x:c>
+      <x:c r="D7" s="10"/>
     </x:row>
     <x:row r="8" ht="64" customHeight="1">
       <x:c r="A8" s="9" t="str">
@@ -1119,6 +1172,7 @@
       <x:c r="C8" s="9" t="str">
         <x:v>Name, Severity, Enabled and Message can be set on the first row.</x:v>
       </x:c>
+      <x:c r="D8" s="10"/>
     </x:row>
     <x:row r="9" ht="64" customHeight="1">
       <x:c r="A9" s="9" t="str">
@@ -1130,6 +1184,7 @@
       <x:c r="C9" s="9" t="str">
         <x:v>Field values must match the exact technical keys from Columns.</x:v>
       </x:c>
+      <x:c r="D9" s="10"/>
     </x:row>
     <x:row r="10" ht="64" customHeight="1">
       <x:c r="A10" s="9" t="str">
@@ -1141,6 +1196,7 @@
       <x:c r="C10" s="9" t="str">
         <x:v>Group root / Join all; Group 1 / Join any</x:v>
       </x:c>
+      <x:c r="D10" s="10"/>
     </x:row>
     <x:row r="11" ht="64" customHeight="1">
       <x:c r="A11" s="9" t="str">
@@ -1152,6 +1208,7 @@
       <x:c r="C11" s="9" t="str">
         <x:v>MOVEMENT_TYPE / eq / 201</x:v>
       </x:c>
+      <x:c r="D11" s="10"/>
     </x:row>
     <x:row r="12" ht="64" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -1163,6 +1220,7 @@
       <x:c r="C12" s="9" t="str">
         <x:v>END_DATE / fieldGte / Other field START_DATE</x:v>
       </x:c>
+      <x:c r="D12" s="10"/>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
       <x:c r="A13" s="9" t="str">
@@ -1174,6 +1232,7 @@
       <x:c r="C13" s="9" t="str">
         <x:v>CONTACT / pattern / email</x:v>
       </x:c>
+      <x:c r="D13" s="10"/>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
       <x:c r="A14" s="9" t="str">
@@ -1185,6 +1244,7 @@
       <x:c r="C14" s="9" t="str">
         <x:v>Separate Description columns with semicolons or newlines.</x:v>
       </x:c>
+      <x:c r="D14" s="10"/>
     </x:row>
     <x:row r="15" ht="64" customHeight="1">
       <x:c r="A15" s="9" t="str">
@@ -1196,6 +1256,7 @@
       <x:c r="C15" s="9" t="str">
         <x:v>PLANT / lookup / plants / Plant</x:v>
       </x:c>
+      <x:c r="D15" s="10"/>
     </x:row>
     <x:row r="16" ht="64" customHeight="1">
       <x:c r="A16" s="9" t="str">
@@ -1207,6 +1268,7 @@
       <x:c r="C16" s="9" t="str">
         <x:v>PLANT=Plant;STORAGE_LOCATION=Storage location</x:v>
       </x:c>
+      <x:c r="D16" s="10"/>
     </x:row>
     <x:row r="17" ht="64" customHeight="1">
       <x:c r="A17" s="9" t="str">
@@ -1218,17 +1280,19 @@
       <x:c r="C17" s="9" t="str">
         <x:v>MATERIAL,PLANT,STORAGE_LOCATION</x:v>
       </x:c>
+      <x:c r="D17" s="10"/>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>Limits</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>Up to 80 columns, 100 rules, 400 when clauses, 20 reference lists and 20 unique combinations. Keep the workbook below 10 MB.</x:v>
+        <x:v>Up to 200 columns, 100 rules, 400 when clauses, 20 reference lists and 20 unique combinations. Keep the workbook below 10 MB.</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
         <x:v>Remove a sheet only when you do not use that section. Template and Columns are required.</x:v>
       </x:c>
+      <x:c r="D18" s="10"/>
     </x:row>
     <x:row r="19" ht="64" customHeight="1">
       <x:c r="A19" s="9" t="str">
@@ -1240,11 +1304,63 @@
       <x:c r="C19" s="9" t="str">
         <x:v>This file configures validation rules. Use the Validate tab for data files to check.</x:v>
       </x:c>
+      <x:c r="D19" s="10"/>
     </x:row>
     <x:row r="20" ht="64" customHeight="1">
-      <x:c r="A20" s="10"/>
-      <x:c r="B20" s="10"/>
-      <x:c r="C20" s="10"/>
+      <x:c r="A20" s="9" t="str">
+        <x:v>Template type</x:v>
+      </x:c>
+      <x:c r="B20" s="9" t="str">
+        <x:v>General preserves the existing checks. For SAP choose SAP in Template, and fill SAP type, SAP length, SAP decimals and optional SAP reference field on Columns. General Type stays text if unused.</x:v>
+      </x:c>
+      <x:c r="C20" s="9" t="str">
+        <x:v>SAP date DATS / 8; currency CURR / 15 / 2 → CUKY field.</x:v>
+      </x:c>
+      <x:c r="D20" s="10"/>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="7" t="str">
+        <x:v>SAP formats</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="str">
+        <x:v>Use internal formats: DATS YYYYMMDD (initial 00000000), TIMS HHMMSS, NUMC fixed digits, signed plain decimals with a dot. No zero padding, rounding or conversion exits are applied.</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="str">
+        <x:v>Keep technical codes and long numbers as Text in Excel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="7" t="str">
+        <x:v>SAP scope</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>18 supported DDIC formats. Use actual SE11 definitions. Domain values, conversion exits and currency display scaling need your system-specific Conditions/References.</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>Source: https://help.sap.com/doc/abapdocu_754_index_htm/7.54/en-US/abenddic_builtin_types.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="7" t="str">
+        <x:v>Simpler option</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>For column setup without Excel conditions/references, use the one-sheet simple General or SAP setup download instead. You can maintain Conditions and References later inside Studio.</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>A single Setup sheet: name in B2, type in B3, fields from row 9.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="7" t="str">
+        <x:v>Upload size</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="str">
+        <x:v>Data validation stays within 5,000 rows and 200,000 cells. At 200 columns, upload up to 1,000 data rows per file.</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="str">
+        <x:v>Setup rows define fields; data rows are uploaded separately on Validate.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Support multiple THEN field requirements per validation condition
</commit_message>
<xml_diff>
--- a/validation-setup-template.xlsx
+++ b/validation-setup-template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R9d5d93231b164856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rdf0e0141df024f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R8efab30ae9544022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R3f97f1e005b14e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R5876b80466544567"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R3f86236627b54cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rd8053f9e33204341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R677617d23d3241ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="Rc4907a6d42d2410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="R17f2810b001144eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="Rf0bc7165b1da42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R4d15dbafa6754bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="Rdb117cff232146c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="Rd24f04d5dda34ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rf01bd43406c544f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R1453e83602d54b28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1167,7 +1167,7 @@
         <x:v>Conditions</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Use one Rule ID for each rule. Each rule needs exactly one assert row. Add when rows under the same ID for the trigger. With no when rows, the rule always applies.</x:v>
+        <x:v>Use one Rule ID per condition. Add one or more assert rows under that ID for THEN requirements; all must pass. Add when rows for the trigger. With no when rows, every record is checked.</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Name, Severity, Enabled and Message can be set on the first row.</x:v>

</xml_diff>

<commit_message>
Allow multiple THEN REQUIRE fields in Validation Studio (#132)
</commit_message>
<xml_diff>
--- a/validation-setup-template.xlsx
+++ b/validation-setup-template.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R9d5d93231b164856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="Rdf0e0141df024f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="R8efab30ae9544022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R3f97f1e005b14e61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="R5876b80466544567"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="R3f86236627b54cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rd8053f9e33204341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R677617d23d3241ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="Rc4907a6d42d2410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" r:id="R17f2810b001144eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditions" sheetId="3" r:id="Rf0bc7165b1da42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="4" r:id="R4d15dbafa6754bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique combinations" sheetId="5" r:id="Rdb117cff232146c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plants" sheetId="6" r:id="Rd24f04d5dda34ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Storage locations" sheetId="7" r:id="Rf01bd43406c544f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="8" r:id="R1453e83602d54b28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1167,7 +1167,7 @@
         <x:v>Conditions</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Use one Rule ID for each rule. Each rule needs exactly one assert row. Add when rows under the same ID for the trigger. With no when rows, the rule always applies.</x:v>
+        <x:v>Use one Rule ID per condition. Add one or more assert rows under that ID for THEN requirements; all must pass. Add when rows for the trigger. With no when rows, every record is checked.</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Name, Severity, Enabled and Message can be set on the first row.</x:v>

</xml_diff>